<commit_message>
Fix conditional formatting so typing X turns cells green
Replaced the broken CellIsRule (which compared against two spaces instead
of an empty string) with a single FormulaRule using LEN(TRIM(...))>0.
This correctly triggers the green fill for any non-blank day cell.

https://claude.ai/code/session_018vCMC1CFJpstUVJpAwWUfd
</commit_message>
<xml_diff>
--- a/Habit_Tracker_April_2026.xlsx
+++ b/Habit_Tracker_April_2026.xlsx
@@ -1696,11 +1696,8 @@
     <mergeCell ref="A1:AI1"/>
   </mergeCells>
   <conditionalFormatting sqref="D4:AG20">
-    <cfRule type="cellIs" priority="1" operator="notEqual" dxfId="0">
-      <formula>"  "</formula>
-    </cfRule>
-    <cfRule type="expression" priority="2" dxfId="0">
-      <formula>D4&lt;&gt;""</formula>
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>LEN(TRIM(D4))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Remove green conditional formatting, keep checkbox dropdowns only
https://claude.ai/code/session_018vCMC1CFJpstUVJpAwWUfd
</commit_message>
<xml_diff>
--- a/Habit_Tracker_April_2026.xlsx
+++ b/Habit_Tracker_April_2026.xlsx
@@ -407,35 +407,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FFFFFFFF"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF5FAD41"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="thin">
-          <color rgb="FFCCCCCC"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFCCCCCC"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFCCCCCC"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFCCCCCC"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
 </styleSheet>
 </file>
@@ -2291,16 +2263,6 @@
     <mergeCell ref="D22:AG22"/>
     <mergeCell ref="D23:AG23"/>
   </mergeCells>
-  <conditionalFormatting sqref="C16:C23">
-    <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
-      <formula>"☑"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C3:AF12">
-    <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
-      <formula>"☑"</formula>
-    </cfRule>
-  </conditionalFormatting>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C3:AF12">
       <formula1>"☑,☐"</formula1>

</xml_diff>

<commit_message>
Use ✓/□ instead of ☑/☐ to avoid Excel 365 auto-green styling
https://claude.ai/code/session_018vCMC1CFJpstUVJpAwWUfd
</commit_message>
<xml_diff>
--- a/Habit_Tracker_April_2026.xlsx
+++ b/Habit_Tracker_April_2026.xlsx
@@ -148,7 +148,7 @@
     <t>Morning Routine</t>
   </si>
   <si>
-    <t>☐</t>
+    <t>□</t>
   </si>
   <si>
     <t>Exercise / Workout</t>
@@ -2265,10 +2265,10 @@
   </mergeCells>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C3:AF12">
-      <formula1>"☑,☐"</formula1>
+      <formula1>"✓,□"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C16:C23">
-      <formula1>"☑,☐"</formula1>
+      <formula1>"✓,□"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Fix progress COUNTIF formula to use updated ✓ character
https://claude.ai/code/session_018vCMC1CFJpstUVJpAwWUfd
</commit_message>
<xml_diff>
--- a/Habit_Tracker_April_2026.xlsx
+++ b/Habit_Tracker_April_2026.xlsx
@@ -936,7 +936,7 @@
         <v>34</v>
       </c>
       <c r="AG3" s="8">
-        <f>COUNTIF(C3:AF3,"☑")/30</f>
+        <f>COUNTIF(C3:AF3,"✓")/30</f>
         <v>0</v>
       </c>
     </row>
@@ -1035,7 +1035,7 @@
         <v>34</v>
       </c>
       <c r="AG4" s="8">
-        <f>COUNTIF(C4:AF4,"☑")/30</f>
+        <f>COUNTIF(C4:AF4,"✓")/30</f>
         <v>0</v>
       </c>
     </row>
@@ -1134,7 +1134,7 @@
         <v>34</v>
       </c>
       <c r="AG5" s="8">
-        <f>COUNTIF(C5:AF5,"☑")/30</f>
+        <f>COUNTIF(C5:AF5,"✓")/30</f>
         <v>0</v>
       </c>
     </row>
@@ -1233,7 +1233,7 @@
         <v>34</v>
       </c>
       <c r="AG6" s="8">
-        <f>COUNTIF(C6:AF6,"☑")/30</f>
+        <f>COUNTIF(C6:AF6,"✓")/30</f>
         <v>0</v>
       </c>
     </row>
@@ -1332,7 +1332,7 @@
         <v>34</v>
       </c>
       <c r="AG7" s="8">
-        <f>COUNTIF(C7:AF7,"☑")/30</f>
+        <f>COUNTIF(C7:AF7,"✓")/30</f>
         <v>0</v>
       </c>
     </row>
@@ -1431,7 +1431,7 @@
         <v>34</v>
       </c>
       <c r="AG8" s="8">
-        <f>COUNTIF(C8:AF8,"☑")/30</f>
+        <f>COUNTIF(C8:AF8,"✓")/30</f>
         <v>0</v>
       </c>
     </row>
@@ -1530,7 +1530,7 @@
         <v>34</v>
       </c>
       <c r="AG9" s="8">
-        <f>COUNTIF(C9:AF9,"☑")/30</f>
+        <f>COUNTIF(C9:AF9,"✓")/30</f>
         <v>0</v>
       </c>
     </row>
@@ -1629,7 +1629,7 @@
         <v>34</v>
       </c>
       <c r="AG10" s="8">
-        <f>COUNTIF(C10:AF10,"☑")/30</f>
+        <f>COUNTIF(C10:AF10,"✓")/30</f>
         <v>0</v>
       </c>
     </row>
@@ -1728,7 +1728,7 @@
         <v>34</v>
       </c>
       <c r="AG11" s="8">
-        <f>COUNTIF(C11:AF11,"☑")/30</f>
+        <f>COUNTIF(C11:AF11,"✓")/30</f>
         <v>0</v>
       </c>
     </row>
@@ -1827,7 +1827,7 @@
         <v>34</v>
       </c>
       <c r="AG12" s="8">
-        <f>COUNTIF(C12:AF12,"☑")/30</f>
+        <f>COUNTIF(C12:AF12,"✓")/30</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix progress formula: count cells not equal to □ instead of equal to ✓
https://claude.ai/code/session_018vCMC1CFJpstUVJpAwWUfd
</commit_message>
<xml_diff>
--- a/Habit_Tracker_April_2026.xlsx
+++ b/Habit_Tracker_April_2026.xlsx
@@ -936,7 +936,7 @@
         <v>34</v>
       </c>
       <c r="AG3" s="8">
-        <f>COUNTIF(C3:AF3,"✓")/30</f>
+        <f>COUNTIF(C3:AF3,"&lt;&gt;□")/30</f>
         <v>0</v>
       </c>
     </row>
@@ -1035,7 +1035,7 @@
         <v>34</v>
       </c>
       <c r="AG4" s="8">
-        <f>COUNTIF(C4:AF4,"✓")/30</f>
+        <f>COUNTIF(C4:AF4,"&lt;&gt;□")/30</f>
         <v>0</v>
       </c>
     </row>
@@ -1134,7 +1134,7 @@
         <v>34</v>
       </c>
       <c r="AG5" s="8">
-        <f>COUNTIF(C5:AF5,"✓")/30</f>
+        <f>COUNTIF(C5:AF5,"&lt;&gt;□")/30</f>
         <v>0</v>
       </c>
     </row>
@@ -1233,7 +1233,7 @@
         <v>34</v>
       </c>
       <c r="AG6" s="8">
-        <f>COUNTIF(C6:AF6,"✓")/30</f>
+        <f>COUNTIF(C6:AF6,"&lt;&gt;□")/30</f>
         <v>0</v>
       </c>
     </row>
@@ -1332,7 +1332,7 @@
         <v>34</v>
       </c>
       <c r="AG7" s="8">
-        <f>COUNTIF(C7:AF7,"✓")/30</f>
+        <f>COUNTIF(C7:AF7,"&lt;&gt;□")/30</f>
         <v>0</v>
       </c>
     </row>
@@ -1431,7 +1431,7 @@
         <v>34</v>
       </c>
       <c r="AG8" s="8">
-        <f>COUNTIF(C8:AF8,"✓")/30</f>
+        <f>COUNTIF(C8:AF8,"&lt;&gt;□")/30</f>
         <v>0</v>
       </c>
     </row>
@@ -1530,7 +1530,7 @@
         <v>34</v>
       </c>
       <c r="AG9" s="8">
-        <f>COUNTIF(C9:AF9,"✓")/30</f>
+        <f>COUNTIF(C9:AF9,"&lt;&gt;□")/30</f>
         <v>0</v>
       </c>
     </row>
@@ -1629,7 +1629,7 @@
         <v>34</v>
       </c>
       <c r="AG10" s="8">
-        <f>COUNTIF(C10:AF10,"✓")/30</f>
+        <f>COUNTIF(C10:AF10,"&lt;&gt;□")/30</f>
         <v>0</v>
       </c>
     </row>
@@ -1728,7 +1728,7 @@
         <v>34</v>
       </c>
       <c r="AG11" s="8">
-        <f>COUNTIF(C11:AF11,"✓")/30</f>
+        <f>COUNTIF(C11:AF11,"&lt;&gt;□")/30</f>
         <v>0</v>
       </c>
     </row>
@@ -1827,7 +1827,7 @@
         <v>34</v>
       </c>
       <c r="AG12" s="8">
-        <f>COUNTIF(C12:AF12,"✓")/30</f>
+        <f>COUNTIF(C12:AF12,"&lt;&gt;□")/30</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Use SUMPRODUCT(EXACT()) for progress formula for reliable Unicode matching
https://claude.ai/code/session_018vCMC1CFJpstUVJpAwWUfd
</commit_message>
<xml_diff>
--- a/Habit_Tracker_April_2026.xlsx
+++ b/Habit_Tracker_April_2026.xlsx
@@ -936,7 +936,7 @@
         <v>34</v>
       </c>
       <c r="AG3" s="8">
-        <f>COUNTIF(C3:AF3,"&lt;&gt;□")/30</f>
+        <f>SUMPRODUCT(EXACT(C3:AF3,"✓"))/30</f>
         <v>0</v>
       </c>
     </row>
@@ -1035,7 +1035,7 @@
         <v>34</v>
       </c>
       <c r="AG4" s="8">
-        <f>COUNTIF(C4:AF4,"&lt;&gt;□")/30</f>
+        <f>SUMPRODUCT(EXACT(C4:AF4,"✓"))/30</f>
         <v>0</v>
       </c>
     </row>
@@ -1134,7 +1134,7 @@
         <v>34</v>
       </c>
       <c r="AG5" s="8">
-        <f>COUNTIF(C5:AF5,"&lt;&gt;□")/30</f>
+        <f>SUMPRODUCT(EXACT(C5:AF5,"✓"))/30</f>
         <v>0</v>
       </c>
     </row>
@@ -1233,7 +1233,7 @@
         <v>34</v>
       </c>
       <c r="AG6" s="8">
-        <f>COUNTIF(C6:AF6,"&lt;&gt;□")/30</f>
+        <f>SUMPRODUCT(EXACT(C6:AF6,"✓"))/30</f>
         <v>0</v>
       </c>
     </row>
@@ -1332,7 +1332,7 @@
         <v>34</v>
       </c>
       <c r="AG7" s="8">
-        <f>COUNTIF(C7:AF7,"&lt;&gt;□")/30</f>
+        <f>SUMPRODUCT(EXACT(C7:AF7,"✓"))/30</f>
         <v>0</v>
       </c>
     </row>
@@ -1431,7 +1431,7 @@
         <v>34</v>
       </c>
       <c r="AG8" s="8">
-        <f>COUNTIF(C8:AF8,"&lt;&gt;□")/30</f>
+        <f>SUMPRODUCT(EXACT(C8:AF8,"✓"))/30</f>
         <v>0</v>
       </c>
     </row>
@@ -1530,7 +1530,7 @@
         <v>34</v>
       </c>
       <c r="AG9" s="8">
-        <f>COUNTIF(C9:AF9,"&lt;&gt;□")/30</f>
+        <f>SUMPRODUCT(EXACT(C9:AF9,"✓"))/30</f>
         <v>0</v>
       </c>
     </row>
@@ -1629,7 +1629,7 @@
         <v>34</v>
       </c>
       <c r="AG10" s="8">
-        <f>COUNTIF(C10:AF10,"&lt;&gt;□")/30</f>
+        <f>SUMPRODUCT(EXACT(C10:AF10,"✓"))/30</f>
         <v>0</v>
       </c>
     </row>
@@ -1728,7 +1728,7 @@
         <v>34</v>
       </c>
       <c r="AG11" s="8">
-        <f>COUNTIF(C11:AF11,"&lt;&gt;□")/30</f>
+        <f>SUMPRODUCT(EXACT(C11:AF11,"✓"))/30</f>
         <v>0</v>
       </c>
     </row>
@@ -1827,7 +1827,7 @@
         <v>34</v>
       </c>
       <c r="AG12" s="8">
-        <f>COUNTIF(C12:AF12,"&lt;&gt;□")/30</f>
+        <f>SUMPRODUCT(EXACT(C12:AF12,"✓"))/30</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Use plain 'x' for checked to avoid Excel 365 auto-checkbox conversion
✓ was being converted to a native boolean by Excel 365, breaking COUNTIF.
Using 'x' avoids auto-formatting and makes COUNTIF reliable.

https://claude.ai/code/session_018vCMC1CFJpstUVJpAwWUfd
</commit_message>
<xml_diff>
--- a/Habit_Tracker_April_2026.xlsx
+++ b/Habit_Tracker_April_2026.xlsx
@@ -936,7 +936,7 @@
         <v>34</v>
       </c>
       <c r="AG3" s="8">
-        <f>SUMPRODUCT(EXACT(C3:AF3,"✓"))/30</f>
+        <f>COUNTIF(C3:AF3,"x")/30</f>
         <v>0</v>
       </c>
     </row>
@@ -1035,7 +1035,7 @@
         <v>34</v>
       </c>
       <c r="AG4" s="8">
-        <f>SUMPRODUCT(EXACT(C4:AF4,"✓"))/30</f>
+        <f>COUNTIF(C4:AF4,"x")/30</f>
         <v>0</v>
       </c>
     </row>
@@ -1134,7 +1134,7 @@
         <v>34</v>
       </c>
       <c r="AG5" s="8">
-        <f>SUMPRODUCT(EXACT(C5:AF5,"✓"))/30</f>
+        <f>COUNTIF(C5:AF5,"x")/30</f>
         <v>0</v>
       </c>
     </row>
@@ -1233,7 +1233,7 @@
         <v>34</v>
       </c>
       <c r="AG6" s="8">
-        <f>SUMPRODUCT(EXACT(C6:AF6,"✓"))/30</f>
+        <f>COUNTIF(C6:AF6,"x")/30</f>
         <v>0</v>
       </c>
     </row>
@@ -1332,7 +1332,7 @@
         <v>34</v>
       </c>
       <c r="AG7" s="8">
-        <f>SUMPRODUCT(EXACT(C7:AF7,"✓"))/30</f>
+        <f>COUNTIF(C7:AF7,"x")/30</f>
         <v>0</v>
       </c>
     </row>
@@ -1431,7 +1431,7 @@
         <v>34</v>
       </c>
       <c r="AG8" s="8">
-        <f>SUMPRODUCT(EXACT(C8:AF8,"✓"))/30</f>
+        <f>COUNTIF(C8:AF8,"x")/30</f>
         <v>0</v>
       </c>
     </row>
@@ -1530,7 +1530,7 @@
         <v>34</v>
       </c>
       <c r="AG9" s="8">
-        <f>SUMPRODUCT(EXACT(C9:AF9,"✓"))/30</f>
+        <f>COUNTIF(C9:AF9,"x")/30</f>
         <v>0</v>
       </c>
     </row>
@@ -1629,7 +1629,7 @@
         <v>34</v>
       </c>
       <c r="AG10" s="8">
-        <f>SUMPRODUCT(EXACT(C10:AF10,"✓"))/30</f>
+        <f>COUNTIF(C10:AF10,"x")/30</f>
         <v>0</v>
       </c>
     </row>
@@ -1728,7 +1728,7 @@
         <v>34</v>
       </c>
       <c r="AG11" s="8">
-        <f>SUMPRODUCT(EXACT(C11:AF11,"✓"))/30</f>
+        <f>COUNTIF(C11:AF11,"x")/30</f>
         <v>0</v>
       </c>
     </row>
@@ -1827,7 +1827,7 @@
         <v>34</v>
       </c>
       <c r="AG12" s="8">
-        <f>SUMPRODUCT(EXACT(C12:AF12,"✓"))/30</f>
+        <f>COUNTIF(C12:AF12,"x")/30</f>
         <v>0</v>
       </c>
     </row>
@@ -2265,10 +2265,10 @@
   </mergeCells>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C3:AF12">
-      <formula1>"✓,□"</formula1>
+      <formula1>"x,□"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C16:C23">
-      <formula1>"✓,□"</formula1>
+      <formula1>"x,□"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>